<commit_message>
Prepare for Vercel + Render deployment
Wire frontend to VITE_API_URL, add Render Procfile/runtime and
Vercel config, and include forecasting + cascading MRP updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/sample_mrp_data.xlsx
+++ b/backend/sample_mrp_data.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Inventory" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Demand_Forecast" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Open_POs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sales_History" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1398,4 +1399,215 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>W-16</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>W-15</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>W-14</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>W-13</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>W-12</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>W-11</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>W-10</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>W-9</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>W-8</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>W-7</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>W-6</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>W-5</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>W-4</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>W-3</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>W-2</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ITM001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H2" t="n">
+        <v>22</v>
+      </c>
+      <c r="I2" t="n">
+        <v>19</v>
+      </c>
+      <c r="J2" t="n">
+        <v>25</v>
+      </c>
+      <c r="K2" t="n">
+        <v>21</v>
+      </c>
+      <c r="L2" t="n">
+        <v>18</v>
+      </c>
+      <c r="M2" t="n">
+        <v>23</v>
+      </c>
+      <c r="N2" t="n">
+        <v>20</v>
+      </c>
+      <c r="O2" t="n">
+        <v>17</v>
+      </c>
+      <c r="P2" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ITM002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G3" t="n">
+        <v>24</v>
+      </c>
+      <c r="H3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I3" t="n">
+        <v>26</v>
+      </c>
+      <c r="J3" t="n">
+        <v>32</v>
+      </c>
+      <c r="K3" t="n">
+        <v>28</v>
+      </c>
+      <c r="L3" t="n">
+        <v>25</v>
+      </c>
+      <c r="M3" t="n">
+        <v>30</v>
+      </c>
+      <c r="N3" t="n">
+        <v>27</v>
+      </c>
+      <c r="O3" t="n">
+        <v>24</v>
+      </c>
+      <c r="P3" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>